<commit_message>
Penambahan permission dan groups
</commit_message>
<xml_diff>
--- a/opensipkd/base/scripts/data/routes.xlsx
+++ b/opensipkd/base/scripts/data/routes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aagus\Project\base\opensipkd\base\scripts\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E55757E2-0E78-490D-877A-CD8349644C35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{630871F0-4B59-4F94-9A3B-E14E0156D94A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{51BF75B7-9F61-46F9-AED2-0C588CFBE466}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="156">
   <si>
     <t>kode</t>
   </si>
@@ -374,7 +374,133 @@
     <t>Partner Uload</t>
   </si>
   <si>
-    <t>W</t>
+    <t>base-permission</t>
+  </si>
+  <si>
+    <t>/permission</t>
+  </si>
+  <si>
+    <t>base-permission-act</t>
+  </si>
+  <si>
+    <t>/permission/{act}/act</t>
+  </si>
+  <si>
+    <t>base-permission-add</t>
+  </si>
+  <si>
+    <t>/permission/add</t>
+  </si>
+  <si>
+    <t>base-permission-edit</t>
+  </si>
+  <si>
+    <t>/permission/{id}/edit</t>
+  </si>
+  <si>
+    <t>base-permission-view</t>
+  </si>
+  <si>
+    <t>/permission/{id}/view</t>
+  </si>
+  <si>
+    <t>base-permission-delete</t>
+  </si>
+  <si>
+    <t>/permission/{id}/delete</t>
+  </si>
+  <si>
+    <t>base-permission-upload</t>
+  </si>
+  <si>
+    <t>/permission/upload</t>
+  </si>
+  <si>
+    <t>Permission</t>
+  </si>
+  <si>
+    <t>Permission Action</t>
+  </si>
+  <si>
+    <t>Permission Add</t>
+  </si>
+  <si>
+    <t>Permission Edit</t>
+  </si>
+  <si>
+    <t>Permission View</t>
+  </si>
+  <si>
+    <t>Permission Delete</t>
+  </si>
+  <si>
+    <t>Permission Uload</t>
+  </si>
+  <si>
+    <t>base-groups</t>
+  </si>
+  <si>
+    <t>/groups</t>
+  </si>
+  <si>
+    <t>groups</t>
+  </si>
+  <si>
+    <t>base-groups-act</t>
+  </si>
+  <si>
+    <t>/groups/{act}/act</t>
+  </si>
+  <si>
+    <t>base-groups-add</t>
+  </si>
+  <si>
+    <t>/groups/add</t>
+  </si>
+  <si>
+    <t>base-groups-edit</t>
+  </si>
+  <si>
+    <t>/groups/{id}/edit</t>
+  </si>
+  <si>
+    <t>base-groups-view</t>
+  </si>
+  <si>
+    <t>/groups/{id}/view</t>
+  </si>
+  <si>
+    <t>base-groups-delete</t>
+  </si>
+  <si>
+    <t>/groups/{id}/delete</t>
+  </si>
+  <si>
+    <t>base-groups-upload</t>
+  </si>
+  <si>
+    <t>/groups/upload</t>
+  </si>
+  <si>
+    <t>Groups</t>
+  </si>
+  <si>
+    <t>Groups Action</t>
+  </si>
+  <si>
+    <t>Groups Add</t>
+  </si>
+  <si>
+    <t>Groups Edit</t>
+  </si>
+  <si>
+    <t>Groups View</t>
+  </si>
+  <si>
+    <t>Groups Delete</t>
+  </si>
+  <si>
+    <t>Groups Uload</t>
   </si>
 </sst>
 </file>
@@ -1236,7 +1362,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07EE843B-4512-436D-B335-2960BD082919}">
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="19.265625" bestFit="1" customWidth="1"/>
@@ -2091,9 +2217,470 @@
         <v>29</v>
       </c>
     </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A25" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="K25" s="1">
+        <v>1</v>
+      </c>
+      <c r="L25" s="1">
+        <v>0</v>
+      </c>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1">
+        <v>1</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="F26" t="s">
+      <c r="A26" t="s">
+        <v>115</v>
+      </c>
+      <c r="B26" t="s">
+        <v>116</v>
+      </c>
+      <c r="C26" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" t="s">
+        <v>7</v>
+      </c>
+      <c r="H26" t="s">
+        <v>93</v>
+      </c>
+      <c r="I26" t="s">
         <v>113</v>
+      </c>
+      <c r="J26" t="s">
+        <v>128</v>
+      </c>
+      <c r="K26">
+        <v>1</v>
+      </c>
+      <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="O26" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>117</v>
+      </c>
+      <c r="B27" t="s">
+        <v>118</v>
+      </c>
+      <c r="C27" t="s">
+        <v>18</v>
+      </c>
+      <c r="D27" t="s">
+        <v>7</v>
+      </c>
+      <c r="H27" t="s">
+        <v>93</v>
+      </c>
+      <c r="I27" t="s">
+        <v>113</v>
+      </c>
+      <c r="J27" t="s">
+        <v>129</v>
+      </c>
+      <c r="K27">
+        <v>1</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="O27" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>119</v>
+      </c>
+      <c r="B28" t="s">
+        <v>120</v>
+      </c>
+      <c r="C28" t="s">
+        <v>18</v>
+      </c>
+      <c r="D28" t="s">
+        <v>7</v>
+      </c>
+      <c r="H28" t="s">
+        <v>93</v>
+      </c>
+      <c r="I28" t="s">
+        <v>113</v>
+      </c>
+      <c r="J28" t="s">
+        <v>130</v>
+      </c>
+      <c r="K28">
+        <v>1</v>
+      </c>
+      <c r="L28">
+        <v>0</v>
+      </c>
+      <c r="O28" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>121</v>
+      </c>
+      <c r="B29" t="s">
+        <v>122</v>
+      </c>
+      <c r="C29" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" t="s">
+        <v>7</v>
+      </c>
+      <c r="H29" t="s">
+        <v>93</v>
+      </c>
+      <c r="I29" t="s">
+        <v>113</v>
+      </c>
+      <c r="J29" t="s">
+        <v>131</v>
+      </c>
+      <c r="K29">
+        <v>1</v>
+      </c>
+      <c r="L29">
+        <v>0</v>
+      </c>
+      <c r="O29" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
+        <v>123</v>
+      </c>
+      <c r="B30" t="s">
+        <v>124</v>
+      </c>
+      <c r="C30" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30" t="s">
+        <v>7</v>
+      </c>
+      <c r="H30" t="s">
+        <v>93</v>
+      </c>
+      <c r="I30" t="s">
+        <v>113</v>
+      </c>
+      <c r="J30" t="s">
+        <v>132</v>
+      </c>
+      <c r="K30">
+        <v>1</v>
+      </c>
+      <c r="L30">
+        <v>0</v>
+      </c>
+      <c r="O30" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
+        <v>125</v>
+      </c>
+      <c r="B31" t="s">
+        <v>126</v>
+      </c>
+      <c r="C31" t="s">
+        <v>18</v>
+      </c>
+      <c r="D31" t="s">
+        <v>7</v>
+      </c>
+      <c r="H31" t="s">
+        <v>93</v>
+      </c>
+      <c r="I31" t="s">
+        <v>113</v>
+      </c>
+      <c r="J31" t="s">
+        <v>133</v>
+      </c>
+      <c r="K31">
+        <v>1</v>
+      </c>
+      <c r="L31">
+        <v>0</v>
+      </c>
+      <c r="O31" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A32" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="K32" s="1">
+        <v>1</v>
+      </c>
+      <c r="L32" s="1">
+        <v>0</v>
+      </c>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1">
+        <v>1</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>137</v>
+      </c>
+      <c r="B33" t="s">
+        <v>138</v>
+      </c>
+      <c r="C33" t="s">
+        <v>18</v>
+      </c>
+      <c r="D33" t="s">
+        <v>136</v>
+      </c>
+      <c r="H33" t="s">
+        <v>93</v>
+      </c>
+      <c r="I33" t="s">
+        <v>134</v>
+      </c>
+      <c r="J33" t="s">
+        <v>150</v>
+      </c>
+      <c r="K33">
+        <v>1</v>
+      </c>
+      <c r="L33">
+        <v>0</v>
+      </c>
+      <c r="O33" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
+        <v>139</v>
+      </c>
+      <c r="B34" t="s">
+        <v>140</v>
+      </c>
+      <c r="C34" t="s">
+        <v>18</v>
+      </c>
+      <c r="D34" t="s">
+        <v>136</v>
+      </c>
+      <c r="H34" t="s">
+        <v>93</v>
+      </c>
+      <c r="I34" t="s">
+        <v>134</v>
+      </c>
+      <c r="J34" t="s">
+        <v>151</v>
+      </c>
+      <c r="K34">
+        <v>1</v>
+      </c>
+      <c r="L34">
+        <v>0</v>
+      </c>
+      <c r="O34" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>141</v>
+      </c>
+      <c r="B35" t="s">
+        <v>142</v>
+      </c>
+      <c r="C35" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" t="s">
+        <v>136</v>
+      </c>
+      <c r="H35" t="s">
+        <v>93</v>
+      </c>
+      <c r="I35" t="s">
+        <v>134</v>
+      </c>
+      <c r="J35" t="s">
+        <v>152</v>
+      </c>
+      <c r="K35">
+        <v>1</v>
+      </c>
+      <c r="L35">
+        <v>0</v>
+      </c>
+      <c r="O35" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A36" t="s">
+        <v>143</v>
+      </c>
+      <c r="B36" t="s">
+        <v>144</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36" t="s">
+        <v>136</v>
+      </c>
+      <c r="H36" t="s">
+        <v>93</v>
+      </c>
+      <c r="I36" t="s">
+        <v>134</v>
+      </c>
+      <c r="J36" t="s">
+        <v>153</v>
+      </c>
+      <c r="K36">
+        <v>1</v>
+      </c>
+      <c r="L36">
+        <v>0</v>
+      </c>
+      <c r="O36" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>145</v>
+      </c>
+      <c r="B37" t="s">
+        <v>146</v>
+      </c>
+      <c r="C37" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" t="s">
+        <v>136</v>
+      </c>
+      <c r="H37" t="s">
+        <v>93</v>
+      </c>
+      <c r="I37" t="s">
+        <v>134</v>
+      </c>
+      <c r="J37" t="s">
+        <v>154</v>
+      </c>
+      <c r="K37">
+        <v>1</v>
+      </c>
+      <c r="L37">
+        <v>0</v>
+      </c>
+      <c r="O37" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
+        <v>147</v>
+      </c>
+      <c r="B38" t="s">
+        <v>148</v>
+      </c>
+      <c r="C38" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" t="s">
+        <v>136</v>
+      </c>
+      <c r="H38" t="s">
+        <v>93</v>
+      </c>
+      <c r="I38" t="s">
+        <v>134</v>
+      </c>
+      <c r="J38" t="s">
+        <v>155</v>
+      </c>
+      <c r="K38">
+        <v>1</v>
+      </c>
+      <c r="L38">
+        <v>0</v>
+      </c>
+      <c r="O38" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement Google OAuth2 user validation and upload logo functionality
</commit_message>
<xml_diff>
--- a/opensipkd/base/scripts/data/routes.xlsx
+++ b/opensipkd/base/scripts/data/routes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aagus\Project\base\opensipkd\base\scripts\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A2B5353-FA2B-4B8A-988C-E6148CBA9500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F479E59-1C64-45DC-A5BB-9722BA9D6E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{51BF75B7-9F61-46F9-AED2-0C588CFBE466}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="166">
   <si>
     <t>kode</t>
   </si>
@@ -501,6 +501,36 @@
   </si>
   <si>
     <t>Groups Uload</t>
+  </si>
+  <si>
+    <t>base-upload-logo</t>
+  </si>
+  <si>
+    <t>Upload Logo</t>
+  </si>
+  <si>
+    <t>googleOauth2</t>
+  </si>
+  <si>
+    <t>Google Oauth2</t>
+  </si>
+  <si>
+    <t>googlesignin</t>
+  </si>
+  <si>
+    <t>/googlesignin</t>
+  </si>
+  <si>
+    <t>GoogleSignIn</t>
+  </si>
+  <si>
+    <t>upload.pt</t>
+  </si>
+  <si>
+    <t>/upload/logo</t>
+  </si>
+  <si>
+    <t>/googleOauth2</t>
   </si>
 </sst>
 </file>
@@ -1362,7 +1392,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07EE843B-4512-436D-B335-2960BD082919}">
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="19.265625" bestFit="1" customWidth="1"/>
@@ -2491,7 +2521,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>137</v>
       </c>
@@ -2523,7 +2553,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>139</v>
       </c>
@@ -2555,7 +2585,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>141</v>
       </c>
@@ -2587,7 +2617,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>143</v>
       </c>
@@ -2619,7 +2649,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>145</v>
       </c>
@@ -2651,7 +2681,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>147</v>
       </c>
@@ -2683,7 +2713,92 @@
         <v>29</v>
       </c>
     </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A39" t="s">
+        <v>156</v>
+      </c>
+      <c r="B39" t="s">
+        <v>164</v>
+      </c>
+      <c r="H39" t="s">
+        <v>93</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="J39" t="s">
+        <v>157</v>
+      </c>
+      <c r="K39">
+        <v>1</v>
+      </c>
+      <c r="L39">
+        <v>0</v>
+      </c>
+      <c r="N39">
+        <v>1</v>
+      </c>
+      <c r="O39" t="s">
+        <v>163</v>
+      </c>
+      <c r="P39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A40" t="s">
+        <v>158</v>
+      </c>
+      <c r="B40" t="s">
+        <v>165</v>
+      </c>
+      <c r="J40" t="s">
+        <v>159</v>
+      </c>
+      <c r="K40">
+        <v>1</v>
+      </c>
+      <c r="L40">
+        <v>1</v>
+      </c>
+      <c r="N40">
+        <v>0</v>
+      </c>
+      <c r="O40" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A41" t="s">
+        <v>160</v>
+      </c>
+      <c r="B41" t="s">
+        <v>161</v>
+      </c>
+      <c r="C41" t="s">
+        <v>18</v>
+      </c>
+      <c r="G41">
+        <v>1</v>
+      </c>
+      <c r="J41" t="s">
+        <v>162</v>
+      </c>
+      <c r="K41">
+        <v>1</v>
+      </c>
+      <c r="L41">
+        <v>1</v>
+      </c>
+      <c r="N41">
+        <v>0</v>
+      </c>
+      <c r="O41" t="s">
+        <v>76</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement JSON-RPC endpoint handling, enhance view configurations, and add API views for user registration and management
</commit_message>
<xml_diff>
--- a/opensipkd/base/scripts/data/routes.xlsx
+++ b/opensipkd/base/scripts/data/routes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aagus\Project\base\opensipkd\base\scripts\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F479E59-1C64-45DC-A5BB-9722BA9D6E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E5B0194-82F5-4C18-8413-AA8FBEAB21D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{51BF75B7-9F61-46F9-AED2-0C588CFBE466}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{51BF75B7-9F61-46F9-AED2-0C588CFBE466}"/>
   </bookViews>
   <sheets>
     <sheet name="routes" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="166">
   <si>
     <t>kode</t>
   </si>
@@ -1393,27 +1393,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07EE843B-4512-436D-B335-2960BD082919}">
   <dimension ref="A1:P41"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.1328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.9296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.1328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.46484375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.1328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.59765625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.59765625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4.06640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.9296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.59765625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="3.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="3.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1463,7 +1463,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1542,7 +1542,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -1615,7 +1615,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>49</v>
       </c>
@@ -1710,6 +1710,9 @@
       <c r="F8" t="s">
         <v>52</v>
       </c>
+      <c r="H8" t="s">
+        <v>43</v>
+      </c>
       <c r="J8" t="s">
         <v>53</v>
       </c>
@@ -1726,7 +1729,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>55</v>
       </c>
@@ -1758,7 +1761,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1793,7 +1796,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>64</v>
       </c>
@@ -1819,7 +1822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>67</v>
       </c>
@@ -1857,7 +1860,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -1889,7 +1892,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -1921,7 +1924,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>81</v>
       </c>
@@ -1953,7 +1956,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>84</v>
       </c>
@@ -1985,7 +1988,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>87</v>
       </c>
@@ -2017,7 +2020,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>90</v>
       </c>
@@ -2055,7 +2058,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>95</v>
       </c>
@@ -2087,7 +2090,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>98</v>
       </c>
@@ -2119,7 +2122,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>101</v>
       </c>
@@ -2151,7 +2154,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>104</v>
       </c>
@@ -2183,7 +2186,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>107</v>
       </c>
@@ -2215,7 +2218,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>110</v>
       </c>
@@ -2247,7 +2250,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>113</v>
       </c>
@@ -2288,7 +2291,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>115</v>
       </c>
@@ -2320,7 +2323,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>117</v>
       </c>
@@ -2352,7 +2355,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>119</v>
       </c>
@@ -2384,7 +2387,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>121</v>
       </c>
@@ -2416,7 +2419,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>123</v>
       </c>
@@ -2448,7 +2451,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>125</v>
       </c>
@@ -2480,7 +2483,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>134</v>
       </c>
@@ -2521,7 +2524,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>137</v>
       </c>
@@ -2553,7 +2556,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>139</v>
       </c>
@@ -2585,7 +2588,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>141</v>
       </c>
@@ -2617,7 +2620,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>143</v>
       </c>
@@ -2649,7 +2652,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>145</v>
       </c>
@@ -2681,7 +2684,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>147</v>
       </c>
@@ -2713,7 +2716,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>156</v>
       </c>
@@ -2745,7 +2748,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>158</v>
       </c>
@@ -2768,7 +2771,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>160</v>
       </c>

</xml_diff>